<commit_message>
#PR 4 - Updated Feature Tickets (#23)
* Resolved merge conflict

* Added ticket automation

* Completed 1 senario in the in the Tickets features

* feature file change

* senario update

* for jenkins

* jenkins proplem solve

* scenario-2 done

* feature 2 completed

* for jenkins

* commanLogins

---------

Co-authored-by: Subathra-subu <subathrasubu2004@gmail.com>
</commit_message>
<xml_diff>
--- a/Cyclos/src/test/resources/testData/ExcelData.xlsx
+++ b/Cyclos/src/test/resources/testData/ExcelData.xlsx
@@ -4,11 +4,12 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="11520" windowHeight="9000" activeTab="1"/>
+    <workbookView windowWidth="11520" windowHeight="9000" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="ExcelData" sheetId="1" r:id="rId1"/>
     <sheet name="AddFeature_sriram_k" sheetId="2" r:id="rId2"/>
+    <sheet name="valid_vovucher" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
   <si>
     <t>name</t>
   </si>
@@ -52,6 +53,33 @@
   </si>
   <si>
     <t>SRIRAM_TITOO</t>
+  </si>
+  <si>
+    <t>voucher code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+6474-7995-6794-5397-3149</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+0495-5575-8604-0009-3516</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+2259-9257-5837-6271-5351</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+3869-3612-1599-4049-2747</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+1069-6165-2688-6425-0159</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+5665-5680-6241-4626-4549</t>
   </si>
 </sst>
 </file>
@@ -667,9 +695,12 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1256,4 +1287,54 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="6"/>
+  <cols>
+    <col min="1" max="1" width="59.8888888888889" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" ht="28.8" spans="1:1">
+      <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" ht="28.8" spans="1:1">
+      <c r="A3" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" ht="28.8" spans="1:1">
+      <c r="A4" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" ht="28.8" spans="1:1">
+      <c r="A5" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" ht="28.8" spans="1:1">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" ht="28.8" spans="1:1">
+      <c r="A7" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Login feature - Excel data updated
</commit_message>
<xml_diff>
--- a/Cyclos/src/test/resources/testData/ExcelData.xlsx
+++ b/Cyclos/src/test/resources/testData/ExcelData.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19200" windowHeight="6200"/>
+    <workbookView windowWidth="19200" windowHeight="6800"/>
   </bookViews>
   <sheets>
     <sheet name="UserLogin_Subathra" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
   <si>
     <t>UserName</t>
   </si>
@@ -37,6 +37,9 @@
   </si>
   <si>
     <t>demo</t>
+  </si>
+  <si>
+    <t>NA</t>
   </si>
   <si>
     <t>name</t>
@@ -73,14 +76,7 @@
     <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
     <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
-  <fonts count="21">
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -553,133 +549,133 @@
     <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -687,7 +683,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1221,8 +1217,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="1"/>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="1"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
@@ -1241,6 +1237,14 @@
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1257,30 +1261,30 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2">
         <v>1</v>

</xml_diff>

<commit_message>
PR1# - Implementation of Login feature (#16)
* Helper,BaseAction,Configure class updated

* Added tag in feature file

* Updated

* Login feature - Excel data updated

---------

Co-authored-by: SRIRAM K <wavene20@gmail.com>
</commit_message>
<xml_diff>
--- a/Cyclos/src/test/resources/testData/ExcelData.xlsx
+++ b/Cyclos/src/test/resources/testData/ExcelData.xlsx
@@ -4,12 +4,11 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="11520" windowHeight="9000" activeTab="2"/>
+    <workbookView windowWidth="19200" windowHeight="6800"/>
   </bookViews>
   <sheets>
-    <sheet name="ExcelData" sheetId="1" r:id="rId1"/>
+    <sheet name="UserLogin_Subathra" sheetId="1" r:id="rId1"/>
     <sheet name="AddFeature_sriram_k" sheetId="2" r:id="rId2"/>
-    <sheet name="valid_vovucher" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -29,7 +28,19 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="15">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+  <si>
+    <t>UserName</t>
+  </si>
+  <si>
+    <t>Password</t>
+  </si>
+  <si>
+    <t>demo</t>
+  </si>
+  <si>
+    <t>NA</t>
+  </si>
   <si>
     <t>name</t>
   </si>
@@ -54,43 +65,16 @@
   <si>
     <t>SRIRAM_TITOO</t>
   </si>
-  <si>
-    <t>voucher code</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-6474-7995-6794-5397-3149</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-0495-5575-8604-0009-3516</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-2259-9257-5837-6271-5351</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-3869-3612-1599-4049-2747</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-1069-6165-2688-6425-0159</t>
-  </si>
-  <si>
-    <t xml:space="preserve">
-5665-5680-6241-4626-4549</t>
-  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
   <numFmts count="4">
-    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
-    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
-    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -553,16 +537,16 @@
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -699,9 +683,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1235,9 +1217,37 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4"/>
-  <sheetData/>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" s="1"/>
+      <c r="B2" s="1">
+        <v>1234</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
 </worksheet>
@@ -1247,90 +1257,40 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="4"/>
+  <sheetFormatPr defaultColWidth="8.89090909090909" defaultRowHeight="14.5" outlineLevelRow="1" outlineLevelCol="4"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="D2">
         <v>1</v>
       </c>
       <c r="E2">
         <v>12</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <headerFooter/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
-  <sheetPr/>
-  <dimension ref="A1:A7"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelRow="6"/>
-  <cols>
-    <col min="1" max="1" width="59.8888888888889" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" ht="28.8" spans="1:1">
-      <c r="A2" s="1" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="3" ht="28.8" spans="1:1">
-      <c r="A3" s="1" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="4" ht="28.8" spans="1:1">
-      <c r="A4" s="1" t="s">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="5" ht="28.8" spans="1:1">
-      <c r="A5" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="6" ht="28.8" spans="1:1">
-      <c r="A6" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="7" ht="28.8" spans="1:1">
-      <c r="A7" s="1" t="s">
-        <v>14</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
enhance the feature with excel and delete scenario
</commit_message>
<xml_diff>
--- a/Cyclos/src/test/resources/testData/ExcelData.xlsx
+++ b/Cyclos/src/test/resources/testData/ExcelData.xlsx
@@ -1,17 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2445" windowWidth="12090" windowHeight="3060"/>
+    <workbookView windowWidth="13128" windowHeight="9000" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="UserLogin_Subathra" sheetId="1" r:id="rId1"/>
     <sheet name="AddFeature_sriram_k" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <oleSize ref="A1:K8"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -70,8 +69,14 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="42" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;_);_(@_)"/>
+    <numFmt numFmtId="44" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -79,16 +84,346 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -96,9 +431,251 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -108,158 +685,89 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
         </patternFill>
       </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
         </patternFill>
       </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <font>
+        <b val="1"/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
+        <b val="1"/>
         <color theme="1"/>
       </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
+        <b val="1"/>
         <color theme="1"/>
       </font>
       <border>
@@ -270,7 +778,7 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
         <color theme="0"/>
       </font>
       <fill>
@@ -298,32 +806,149 @@
           <color theme="4"/>
         </bottom>
         <horizontal style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
+          <color theme="4" tint="0.399975585192419"/>
         </horizontal>
       </border>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
-      <tableStyleElement type="wholeTable" dxfId="16"/>
-      <tableStyleElement type="headerRow" dxfId="15"/>
-      <tableStyleElement type="totalRow" dxfId="14"/>
-      <tableStyleElement type="firstColumn" dxfId="13"/>
-      <tableStyleElement type="lastColumn" dxfId="12"/>
-      <tableStyleElement type="firstRowStripe" dxfId="11"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="10"/>
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
+      <tableStyleElement type="wholeTable" dxfId="6"/>
+      <tableStyleElement type="headerRow" dxfId="5"/>
+      <tableStyleElement type="totalRow" dxfId="4"/>
+      <tableStyleElement type="firstColumn" dxfId="3"/>
+      <tableStyleElement type="lastColumn" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
-      <tableStyleElement type="headerRow" dxfId="9"/>
-      <tableStyleElement type="totalRow" dxfId="8"/>
-      <tableStyleElement type="firstRowStripe" dxfId="7"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="6"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="5"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="4"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="3"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="2"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="1"/>
-      <tableStyleElement type="pageFieldValues" dxfId="0"/>
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
+      <tableStyleElement type="headerRow" dxfId="16"/>
+      <tableStyleElement type="totalRow" dxfId="15"/>
+      <tableStyleElement type="firstRowStripe" dxfId="14"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
+      <tableStyleElement type="pageFieldValues" dxfId="7"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -586,14 +1211,14 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4" outlineLevelRow="3" outlineLevelCol="1"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
@@ -624,13 +1249,15 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85185185185185" defaultRowHeight="14.4" outlineLevelRow="1" outlineLevelCol="4"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
@@ -668,5 +1295,6 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: complete payment request functionality with print and validation workflows
</commit_message>
<xml_diff>
--- a/Cyclos/src/test/resources/testData/ExcelData.xlsx
+++ b/Cyclos/src/test/resources/testData/ExcelData.xlsx
@@ -1,35 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\cyclos_init\Cyclos_AutomationTesting\Cyclos\src\test\resources\testData\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7BC578E-8BE3-4D59-B08D-B304A40960E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2445" windowWidth="12090" windowHeight="2625"/>
+    <workbookView xWindow="4668" yWindow="3360" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserLogin_Subathra" sheetId="1" r:id="rId1"/>
     <sheet name="AddFeature_sriram_k" sheetId="2" r:id="rId2"/>
+    <sheet name="PaymentRequest_Krishna" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:K7"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
     <t>UserName</t>
   </si>
@@ -65,18 +58,52 @@
   </si>
   <si>
     <t>SRIRAM_TITOO</t>
+  </si>
+  <si>
+    <t>Receiver</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Car repair</t>
+  </si>
+  <si>
+    <t>100,00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -97,18 +124,31 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="17">
@@ -304,7 +344,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="16"/>
       <tableStyleElement type="headerRow" dxfId="15"/>
       <tableStyleElement type="totalRow" dxfId="14"/>
@@ -313,7 +353,7 @@
       <tableStyleElement type="firstRowStripe" dxfId="11"/>
       <tableStyleElement type="firstColumnStripe" dxfId="10"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
       <tableStyleElement type="headerRow" dxfId="9"/>
       <tableStyleElement type="totalRow" dxfId="8"/>
       <tableStyleElement type="firstRowStripe" dxfId="7"/>
@@ -329,6 +369,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -591,9 +634,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
@@ -628,9 +671,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
@@ -669,4 +712,37 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F00A3B86-C071-41EF-A5CB-BCF14577C93F}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="3"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" display="https://demo.cyclos.org/ui/" xr:uid="{C69975D6-FA9B-4DCE-86D0-FBD6EC87E2F9}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
feat: complete payment request functionality with print and validation workflows (#53)
</commit_message>
<xml_diff>
--- a/Cyclos/src/test/resources/testData/ExcelData.xlsx
+++ b/Cyclos/src/test/resources/testData/ExcelData.xlsx
@@ -1,35 +1,28 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\cyclos_init\Cyclos_AutomationTesting\Cyclos\src\test\resources\testData\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E7BC578E-8BE3-4D59-B08D-B304A40960E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2445" windowWidth="12090" windowHeight="2625"/>
+    <workbookView xWindow="4668" yWindow="3360" windowWidth="17280" windowHeight="8880" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="UserLogin_Subathra" sheetId="1" r:id="rId1"/>
     <sheet name="AddFeature_sriram_k" sheetId="2" r:id="rId2"/>
+    <sheet name="PaymentRequest_Krishna" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:K7"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
     <t>UserName</t>
   </si>
@@ -65,18 +58,52 @@
   </si>
   <si>
     <t>SRIRAM_TITOO</t>
+  </si>
+  <si>
+    <t>Receiver</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Car repair</t>
+  </si>
+  <si>
+    <t>100,00</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -97,18 +124,31 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="17">
@@ -304,7 +344,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="16"/>
       <tableStyleElement type="headerRow" dxfId="15"/>
       <tableStyleElement type="totalRow" dxfId="14"/>
@@ -313,7 +353,7 @@
       <tableStyleElement type="firstRowStripe" dxfId="11"/>
       <tableStyleElement type="firstColumnStripe" dxfId="10"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
       <tableStyleElement type="headerRow" dxfId="9"/>
       <tableStyleElement type="totalRow" dxfId="8"/>
       <tableStyleElement type="firstRowStripe" dxfId="7"/>
@@ -329,6 +369,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -591,9 +634,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="1" t="s">
@@ -628,9 +671,9 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
@@ -669,4 +712,37 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F00A3B86-C071-41EF-A5CB-BCF14577C93F}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="3" max="3" width="10.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>12</v>
+      </c>
+      <c r="B1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="C2" s="3"/>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="A2" r:id="rId1" display="https://demo.cyclos.org/ui/" xr:uid="{C69975D6-FA9B-4DCE-86D0-FBD6EC87E2F9}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
PR#10Business directory shobana (#68)
* Added Business Directory

* Added

* Added feature 2

* added

* excel added

* Added

* Added tag for feature

* Update testng.xml

* Fix XML structure by closing test and suite tags

* Update ReqpaymentActions.java

* Update PaymentRequestPage.java

* Update PaymentRequestSteps.java
</commit_message>
<xml_diff>
--- a/Cyclos/src/test/resources/testData/ExcelData.xlsx
+++ b/Cyclos/src/test/resources/testData/ExcelData.xlsx
@@ -4,16 +4,16 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2445" windowWidth="12090" windowHeight="2625" firstSheet="2" activeTab="2"/>
+    <workbookView xWindow="0" yWindow="2445" windowWidth="12090" windowHeight="3060" activeTab="2"/>
   </bookViews>
   <sheets>
-    <sheet name="UserLogin_Subathra" sheetId="1" r:id="rId1"/>
+    <sheet name="ExcelData" sheetId="1" r:id="rId1"/>
     <sheet name="AddFeature_sriram_k" sheetId="2" r:id="rId2"/>
-    <sheet name="businessDirectory_shobana" sheetId="3" r:id="rId3"/>
-    <sheet name="favourites_akkshee" sheetId="4" r:id="rId4"/>
+    <sheet name="valid_vovucher" sheetId="3" r:id="rId3"/>
+    <sheet name="businessDirectory" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:L7"/>
+  <oleSize ref="A1:G5"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -31,19 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
-  <si>
-    <t>UserName</t>
-  </si>
-  <si>
-    <t>Password</t>
-  </si>
-  <si>
-    <t>demo</t>
-  </si>
-  <si>
-    <t>NA</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>name</t>
   </si>
@@ -69,10 +57,31 @@
     <t>SRIRAM_TITOO</t>
   </si>
   <si>
-    <t>favourites</t>
-  </si>
-  <si>
-    <t>5 star</t>
+    <t>voucher code</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+6474-7995-6794-5397-3149</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+0495-5575-8604-0009-3516</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+2259-9257-5837-6271-5351</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+3869-3612-1599-4049-2747</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+1069-6165-2688-6425-0159</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+5665-5680-6241-4626-4549</t>
   </si>
   <si>
     <t>keyword</t>
@@ -120,7 +129,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -606,37 +617,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="10" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1">
-        <v>1234</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
-        <v>3</v>
-      </c>
-      <c r="B4" t="s">
-        <v>3</v>
-      </c>
-    </row>
-  </sheetData>
+  <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -648,30 +631,30 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" t="s">
         <v>4</v>
-      </c>
-      <c r="B1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E1" t="s">
-        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>9</v>
+        <v>5</v>
       </c>
       <c r="B2" t="s">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="C2" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -687,21 +670,49 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="59.85546875" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1" ht="30">
+      <c r="A2" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="30">
+      <c r="A3" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" ht="30">
+      <c r="A4" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1" ht="30">
+      <c r="A5" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" ht="30">
+      <c r="A6" s="1" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1" ht="30">
+      <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:1">
-      <c r="A2" t="s">
-        <v>15</v>
-      </c>
-    </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -712,12 +723,12 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
QA: Update payment request test data and empty date scenario
</commit_message>
<xml_diff>
--- a/Cyclos/src/test/resources/testData/ExcelData.xlsx
+++ b/Cyclos/src/test/resources/testData/ExcelData.xlsx
@@ -1,37 +1,30 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30228"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\cyclos_init\Cyclos_AutomationTesting\Cyclos\src\test\resources\testData\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{067F3C35-5656-413C-AAD7-A58B6B06365E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2445" windowWidth="12090" windowHeight="2850" firstSheet="1" activeTab="3"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="1" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ExcelData" sheetId="1" r:id="rId1"/>
     <sheet name="AddFeature_sriram_k" sheetId="2" r:id="rId2"/>
     <sheet name="valid_vovucher" sheetId="3" r:id="rId3"/>
     <sheet name="businessDirectory" sheetId="4" r:id="rId4"/>
+    <sheet name="PaymentRequest_Krishna" sheetId="5" r:id="rId5"/>
   </sheets>
   <calcPr calcId="0"/>
-  <oleSize ref="A1:L8"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>name</t>
   </si>
@@ -89,11 +82,20 @@
   <si>
     <t>pool</t>
   </si>
+  <si>
+    <t>Receiver</t>
+  </si>
+  <si>
+    <t>Amount</t>
+  </si>
+  <si>
+    <t>Active Walking</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
   <fonts count="1">
     <font>
       <sz val="11"/>
@@ -329,7 +331,7 @@
     </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{00000000-0011-0000-FFFF-FFFF00000000}">
       <tableStyleElement type="wholeTable" dxfId="16"/>
       <tableStyleElement type="headerRow" dxfId="15"/>
       <tableStyleElement type="totalRow" dxfId="14"/>
@@ -338,7 +340,7 @@
       <tableStyleElement type="firstRowStripe" dxfId="11"/>
       <tableStyleElement type="firstColumnStripe" dxfId="10"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{00000000-0011-0000-FFFF-FFFF01000000}">
       <tableStyleElement type="headerRow" dxfId="9"/>
       <tableStyleElement type="totalRow" dxfId="8"/>
       <tableStyleElement type="firstRowStripe" dxfId="7"/>
@@ -354,6 +356,9 @@
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
       <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
     </ext>
   </extLst>
 </styleSheet>
@@ -616,18 +621,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.4"/>
   <sheetData/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
@@ -669,11 +674,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:A7"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="59.85546875" customWidth="1"/>
+    <col min="1" max="1" width="59.88671875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
@@ -681,32 +686,32 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="30">
+    <row r="2" spans="1:1" ht="28.8">
       <c r="A2" s="1" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="30">
+    <row r="3" spans="1:1" ht="28.8">
       <c r="A3" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="30">
+    <row r="4" spans="1:1" ht="28.8">
       <c r="A4" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="30">
+    <row r="5" spans="1:1" ht="28.8">
       <c r="A5" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="30">
+    <row r="6" spans="1:1" ht="28.8">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="30">
+    <row r="7" spans="1:1" ht="28.8">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -717,9 +722,9 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
@@ -734,4 +739,30 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1DF1481A-6A7D-4900-AA59-5C81C0A1146A}">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>17</v>
+      </c>
+      <c r="B1" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
PR#15 - Updated Excel data for Invalid login scenarios (#108)
* Fix merge conflict in testng.xml

Removed merge conflict markers from testng.xml

* Update Cucumber feature path in TestNGRunner

* Message feature - scenario added

* conflicts resolved

* Add tags for TestNG runner

* .gitignore added

* Updated runner and feature files

* Altered the Messages.feature related files

* Add tags for TestNG runner configuration

* Resolve conflicts

* Resolve conflicts

* Merge branch 'USER_LOGIN_Subathra' of
https://github.com/Subathra-subu/Cyclos_AutomationTesting.git into
USER_LOGIN_Subathra

* Add tags for TestNG runner

* Added one scenario in Message feature

* Updated Exceldata

* Updated Exceldata
</commit_message>
<xml_diff>
--- a/Cyclos/src/test/resources/testData/ExcelData.xlsx
+++ b/Cyclos/src/test/resources/testData/ExcelData.xlsx
@@ -1,19 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9302"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2445" windowWidth="11430" windowHeight="2505" firstSheet="2" activeTab="3"/>
+    <workbookView windowWidth="19200" windowHeight="6800" firstSheet="2"/>
   </bookViews>
   <sheets>
-    <sheet name="ExcelData" sheetId="1" r:id="rId1"/>
+    <sheet name="LoginData" sheetId="1" r:id="rId1"/>
     <sheet name="AddFeature_sriram_k" sheetId="2" r:id="rId2"/>
     <sheet name="valid_vovucher" sheetId="3" r:id="rId3"/>
     <sheet name="businessDirectory" sheetId="4" r:id="rId4"/>
   </sheets>
-  <calcPr calcId="0"/>
-  <oleSize ref="A1:K6"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -31,7 +30,16 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+  <si>
+    <t>username</t>
+  </si>
+  <si>
+    <t>password</t>
+  </si>
+  <si>
+    <t>demo</t>
+  </si>
   <si>
     <t>name</t>
   </si>
@@ -93,8 +101,14 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <fonts count="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
+  <numFmts count="4">
+    <numFmt numFmtId="176" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="177" formatCode="_ &quot;₹&quot;* #,##0.00_ ;_ &quot;₹&quot;* \-#,##0.00_ ;_ &quot;₹&quot;* &quot;-&quot;??_ ;_ @_ "/>
+    <numFmt numFmtId="178" formatCode="_ * #,##0_ ;_ * \-#,##0_ ;_ * &quot;-&quot;_ ;_ @_ "/>
+    <numFmt numFmtId="179" formatCode="_ &quot;₹&quot;* #,##0_ ;_ &quot;₹&quot;* \-#,##0_ ;_ &quot;₹&quot;* &quot;-&quot;_ ;_ @_ "/>
+  </numFmts>
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -102,16 +116,346 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF0000FF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color rgb="FF800080"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color rgb="FF7F7F7F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="15"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="13"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="3"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF3F3F76"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF3F3F3F"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFA7D00"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C0006"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <charset val="0"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="33">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFCC"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFCC99"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF2F2F2"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFA5A5A5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFC6EFCE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC7CE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.799981688894314"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.399975585192419"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -119,9 +463,251 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFB2B2B2"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFB2B2B2"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFB2B2B2"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFB2B2B2"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="medium">
+        <color theme="4" tint="0.499984740745262"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF7F7F7F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF7F7F7F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF7F7F7F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF7F7F7F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="double">
+        <color rgb="FF3F3F3F"/>
+      </left>
+      <right style="double">
+        <color rgb="FF3F3F3F"/>
+      </right>
+      <top style="double">
+        <color rgb="FF3F3F3F"/>
+      </top>
+      <bottom style="double">
+        <color rgb="FF3F3F3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="double">
+        <color rgb="FFFF8001"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4"/>
+      </top>
+      <bottom style="double">
+        <color theme="4"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="177" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="178" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="179" fontId="0" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -133,158 +719,89 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="49">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Comma" xfId="1" builtinId="3"/>
+    <cellStyle name="Currency" xfId="2" builtinId="4"/>
+    <cellStyle name="Percent" xfId="3" builtinId="5"/>
+    <cellStyle name="Comma [0]" xfId="4" builtinId="6"/>
+    <cellStyle name="Currency [0]" xfId="5" builtinId="7"/>
+    <cellStyle name="Link" xfId="6" builtinId="8"/>
+    <cellStyle name="Followed Hyperlink" xfId="7" builtinId="9"/>
+    <cellStyle name="Note" xfId="8" builtinId="10"/>
+    <cellStyle name="Warning Text" xfId="9" builtinId="11"/>
+    <cellStyle name="Title" xfId="10" builtinId="15"/>
+    <cellStyle name="Explanatory Text" xfId="11" builtinId="53"/>
+    <cellStyle name="Heading 1" xfId="12" builtinId="16"/>
+    <cellStyle name="Heading 2" xfId="13" builtinId="17"/>
+    <cellStyle name="Heading 3" xfId="14" builtinId="18"/>
+    <cellStyle name="Heading 4" xfId="15" builtinId="19"/>
+    <cellStyle name="Input" xfId="16" builtinId="20"/>
+    <cellStyle name="Output" xfId="17" builtinId="21"/>
+    <cellStyle name="Calculation" xfId="18" builtinId="22"/>
+    <cellStyle name="Check Cell" xfId="19" builtinId="23"/>
+    <cellStyle name="Linked Cell" xfId="20" builtinId="24"/>
+    <cellStyle name="Total" xfId="21" builtinId="25"/>
+    <cellStyle name="Good" xfId="22" builtinId="26"/>
+    <cellStyle name="Bad" xfId="23" builtinId="27"/>
+    <cellStyle name="Neutral" xfId="24" builtinId="28"/>
+    <cellStyle name="Accent1" xfId="25" builtinId="29"/>
+    <cellStyle name="20% - Accent1" xfId="26" builtinId="30"/>
+    <cellStyle name="40% - Accent1" xfId="27" builtinId="31"/>
+    <cellStyle name="60% - Accent1" xfId="28" builtinId="32"/>
+    <cellStyle name="Accent2" xfId="29" builtinId="33"/>
+    <cellStyle name="20% - Accent2" xfId="30" builtinId="34"/>
+    <cellStyle name="40% - Accent2" xfId="31" builtinId="35"/>
+    <cellStyle name="60% - Accent2" xfId="32" builtinId="36"/>
+    <cellStyle name="Accent3" xfId="33" builtinId="37"/>
+    <cellStyle name="20% - Accent3" xfId="34" builtinId="38"/>
+    <cellStyle name="40% - Accent3" xfId="35" builtinId="39"/>
+    <cellStyle name="60% - Accent3" xfId="36" builtinId="40"/>
+    <cellStyle name="Accent4" xfId="37" builtinId="41"/>
+    <cellStyle name="20% - Accent4" xfId="38" builtinId="42"/>
+    <cellStyle name="40% - Accent4" xfId="39" builtinId="43"/>
+    <cellStyle name="60% - Accent4" xfId="40" builtinId="44"/>
+    <cellStyle name="Accent5" xfId="41" builtinId="45"/>
+    <cellStyle name="20% - Accent5" xfId="42" builtinId="46"/>
+    <cellStyle name="40% - Accent5" xfId="43" builtinId="47"/>
+    <cellStyle name="60% - Accent5" xfId="44" builtinId="48"/>
+    <cellStyle name="Accent6" xfId="45" builtinId="49"/>
+    <cellStyle name="20% - Accent6" xfId="46" builtinId="50"/>
+    <cellStyle name="40% - Accent6" xfId="47" builtinId="51"/>
+    <cellStyle name="60% - Accent6" xfId="48" builtinId="52"/>
   </cellStyles>
   <dxfs count="17">
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
         </patternFill>
       </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-      </font>
+    </dxf>
+    <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
         </patternFill>
       </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <font>
+        <b val="1"/>
         <color theme="1"/>
       </font>
     </dxf>
     <dxf>
       <font>
+        <b val="1"/>
         <color theme="1"/>
       </font>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
     </dxf>
     <dxf>
       <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-      <border>
-        <top style="thin">
-          <color theme="4"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-      <border>
-        <top style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-      <border>
-        <bottom style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4" tint="0.79995117038483843"/>
-          <bgColor theme="4" tint="0.79995117038483843"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <color theme="1"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
+        <b val="1"/>
         <color theme="1"/>
       </font>
       <border>
@@ -295,7 +812,7 @@
     </dxf>
     <dxf>
       <font>
-        <b/>
+        <b val="1"/>
         <color theme="0"/>
       </font>
       <fill>
@@ -323,32 +840,149 @@
           <color theme="4"/>
         </bottom>
         <horizontal style="thin">
-          <color theme="4" tint="0.39994506668294322"/>
+          <color theme="4" tint="0.399975585192419"/>
         </horizontal>
       </border>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="1"/>
+      </font>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <border>
+        <top style="thin">
+          <color theme="4"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <top style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="1"/>
+        <color theme="1"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4" tint="0.799981688894314"/>
+          <bgColor theme="4" tint="0.799981688894314"/>
+        </patternFill>
+      </fill>
+      <border>
+        <bottom style="thin">
+          <color theme="4" tint="0.399975585192419"/>
+        </bottom>
+      </border>
+    </dxf>
   </dxfs>
   <tableStyles count="2" defaultTableStyle="TableStylePreset3_Accent1" defaultPivotStyle="PivotStylePreset2_Accent1">
-    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7">
-      <tableStyleElement type="wholeTable" dxfId="16"/>
-      <tableStyleElement type="headerRow" dxfId="15"/>
-      <tableStyleElement type="totalRow" dxfId="14"/>
-      <tableStyleElement type="firstColumn" dxfId="13"/>
-      <tableStyleElement type="lastColumn" dxfId="12"/>
-      <tableStyleElement type="firstRowStripe" dxfId="11"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="10"/>
+    <tableStyle name="TableStylePreset3_Accent1" pivot="0" count="7" xr9:uid="{59DB682C-5494-4EDE-A608-00C9E5F0F923}">
+      <tableStyleElement type="wholeTable" dxfId="6"/>
+      <tableStyleElement type="headerRow" dxfId="5"/>
+      <tableStyleElement type="totalRow" dxfId="4"/>
+      <tableStyleElement type="firstColumn" dxfId="3"/>
+      <tableStyleElement type="lastColumn" dxfId="2"/>
+      <tableStyleElement type="firstRowStripe" dxfId="1"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="0"/>
     </tableStyle>
-    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10">
-      <tableStyleElement type="headerRow" dxfId="9"/>
-      <tableStyleElement type="totalRow" dxfId="8"/>
-      <tableStyleElement type="firstRowStripe" dxfId="7"/>
-      <tableStyleElement type="firstColumnStripe" dxfId="6"/>
-      <tableStyleElement type="firstSubtotalRow" dxfId="5"/>
-      <tableStyleElement type="secondSubtotalRow" dxfId="4"/>
-      <tableStyleElement type="firstRowSubheading" dxfId="3"/>
-      <tableStyleElement type="secondRowSubheading" dxfId="2"/>
-      <tableStyleElement type="pageFieldLabels" dxfId="1"/>
-      <tableStyleElement type="pageFieldValues" dxfId="0"/>
+    <tableStyle name="PivotStylePreset2_Accent1" table="0" count="10" xr9:uid="{267968C8-6FFD-4C36-ACC1-9EA1FD1885CA}">
+      <tableStyleElement type="headerRow" dxfId="16"/>
+      <tableStyleElement type="totalRow" dxfId="15"/>
+      <tableStyleElement type="firstRowStripe" dxfId="14"/>
+      <tableStyleElement type="firstColumnStripe" dxfId="13"/>
+      <tableStyleElement type="firstSubtotalRow" dxfId="12"/>
+      <tableStyleElement type="secondSubtotalRow" dxfId="11"/>
+      <tableStyleElement type="firstRowSubheading" dxfId="10"/>
+      <tableStyleElement type="secondRowSubheading" dxfId="9"/>
+      <tableStyleElement type="pageFieldLabels" dxfId="8"/>
+      <tableStyleElement type="pageFieldValues" dxfId="7"/>
     </tableStyle>
   </tableStyles>
   <extLst>
@@ -611,50 +1245,71 @@
     </a:fmtScheme>
   </a:themeElements>
   <a:objectDefaults/>
-  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="15"/>
-  <sheetData/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
+  <dimension ref="A1:B3"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="1"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="B2">
+        <v>1234</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="1" outlineLevelCol="4"/>
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="B1" t="s">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="B2" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C2" t="s">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -665,73 +1320,78 @@
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:A7"/>
-  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="8.85454545454546" defaultRowHeight="14.5" outlineLevelRow="6"/>
   <cols>
-    <col min="1" max="1" width="59.85546875" customWidth="1"/>
+    <col min="1" max="1" width="59.8545454545455" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>11</v>
       </c>
     </row>
-    <row r="2" spans="1:1" ht="30">
+    <row r="2" ht="29" spans="1:1">
       <c r="A2" s="1" t="s">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="30">
+    <row r="3" ht="29" spans="1:1">
       <c r="A3" s="1" t="s">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="30">
+    <row r="4" ht="29" spans="1:1">
       <c r="A4" s="1" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="30">
+    <row r="5" ht="29" spans="1:1">
       <c r="A5" s="1" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="30">
+    <row r="6" ht="29" spans="1:1">
       <c r="A6" s="1" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="30">
+    <row r="7" ht="29" spans="1:1">
       <c r="A7" s="1" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <headerFooter/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
+  <sheetPr/>
   <dimension ref="A1:A2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.5" outlineLevelRow="1"/>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <headerFooter/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Updated Exceldata for blank username and password
</commit_message>
<xml_diff>
--- a/Cyclos/src/test/resources/testData/ExcelData.xlsx
+++ b/Cyclos/src/test/resources/testData/ExcelData.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>username</t>
   </si>
@@ -39,6 +39,9 @@
   </si>
   <si>
     <t>demo</t>
+  </si>
+  <si>
+    <t>NA</t>
   </si>
   <si>
     <t>name</t>
@@ -1251,8 +1254,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="1"/>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="1"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
@@ -1270,6 +1273,14 @@
     <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1286,30 +1297,30 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -1335,37 +1346,37 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" ht="29" spans="1:1">
       <c r="A2" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" ht="29" spans="1:1">
       <c r="A3" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" ht="29" spans="1:1">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" ht="29" spans="1:1">
       <c r="A5" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" ht="29" spans="1:1">
       <c r="A6" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" ht="29" spans="1:1">
       <c r="A7" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1382,12 +1393,12 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
PR#16 - Implementation of filter validation scenario of user in messages feature (#110)
* Fix merge conflict in testng.xml

Removed merge conflict markers from testng.xml

* Update Cucumber feature path in TestNGRunner

* Message feature - scenario added

* conflicts resolved

* Add tags for TestNG runner

* .gitignore added

* Updated runner and feature files

* Altered the Messages.feature related files

* Add tags for TestNG runner configuration

* Resolve conflicts

* Resolve conflicts

* Merge branch 'USER_LOGIN_Subathra' of
https://github.com/Subathra-subu/Cyclos_AutomationTesting.git into
USER_LOGIN_Subathra

* Add tags for TestNG runner

* Added one scenario in Message feature

* Updated Exceldata

* Updated Exceldata

* Updated Exceldata for blank username and password

* Added tag in runner class

* Add message user filter validation

* Resolve merge conflicts

* Resolve wait problems in the filter scenario

* Updation in base actoin
</commit_message>
<xml_diff>
--- a/Cyclos/src/test/resources/testData/ExcelData.xlsx
+++ b/Cyclos/src/test/resources/testData/ExcelData.xlsx
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="21">
   <si>
     <t>username</t>
   </si>
@@ -39,6 +39,9 @@
   </si>
   <si>
     <t>demo</t>
+  </si>
+  <si>
+    <t>NA</t>
   </si>
   <si>
     <t>name</t>
@@ -1251,8 +1254,8 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B3"/>
-  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.5" outlineLevelRow="2" outlineLevelCol="1"/>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr defaultColWidth="10" defaultRowHeight="14.5" outlineLevelRow="3" outlineLevelCol="1"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
@@ -1270,6 +1273,14 @@
     <row r="3" spans="1:2">
       <c r="A3" t="s">
         <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -1286,30 +1297,30 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B1" t="s">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E1" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B2" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="C2" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -1335,37 +1346,37 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="2" ht="29" spans="1:1">
       <c r="A2" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="3" ht="29" spans="1:1">
       <c r="A3" s="1" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="4" ht="29" spans="1:1">
       <c r="A4" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="5" ht="29" spans="1:1">
       <c r="A5" s="1" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6" ht="29" spans="1:1">
       <c r="A6" s="1" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="7" ht="29" spans="1:1">
       <c r="A7" s="1" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>
@@ -1382,12 +1393,12 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
   </sheetData>

</xml_diff>